<commit_message>
Improve dashboard, report, README and SQL
</commit_message>
<xml_diff>
--- a/Ecommerce_Dashboard.xlsx
+++ b/Ecommerce_Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhin\OneDrive\Desktop\Data Analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhin\OneDrive\Desktop\Data Analytics\Indian E-Commerce Sales Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC3E6CA-70F7-4861-BCA1-7CE24307EA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A3A8DB-CFB9-40AA-98FE-E972C08BEBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{FA114D4D-8A45-4CAC-B495-F07891FBDAC8}"/>
   </bookViews>
@@ -37,36 +37,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
   <si>
-    <t>beleza_saude</t>
-  </si>
-  <si>
-    <t>relogios_presentes</t>
-  </si>
-  <si>
-    <t>esporte_lazer</t>
-  </si>
-  <si>
-    <t>cama_mesa_banho</t>
-  </si>
-  <si>
-    <t>informatica_acessorios</t>
-  </si>
-  <si>
-    <t>moveis_decoracao</t>
-  </si>
-  <si>
-    <t>utilidades_domesticas</t>
-  </si>
-  <si>
-    <t>cool_stuff</t>
-  </si>
-  <si>
-    <t>automotivo</t>
-  </si>
-  <si>
-    <t>brinquedos</t>
-  </si>
-  <si>
     <t>product_category_name</t>
   </si>
   <si>
@@ -178,75 +148,6 @@
     <t>total_orders</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>RJ</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>SC</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>RS</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>BA</t>
-  </si>
-  <si>
-    <t>TO</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>SE</t>
-  </si>
-  <si>
-    <t>GO</t>
-  </si>
-  <si>
-    <t>MT</t>
-  </si>
-  <si>
-    <t>MS</t>
-  </si>
-  <si>
-    <t>DF</t>
-  </si>
-  <si>
-    <t>PE</t>
-  </si>
-  <si>
-    <t>PA</t>
-  </si>
-  <si>
-    <t>PB</t>
-  </si>
-  <si>
-    <t>ES</t>
-  </si>
-  <si>
-    <t>AL</t>
-  </si>
-  <si>
-    <t>AM</t>
-  </si>
-  <si>
-    <t>RN</t>
-  </si>
-  <si>
-    <t>RO</t>
-  </si>
-  <si>
     <t>customer_state</t>
   </si>
   <si>
@@ -277,9 +178,6 @@
     <t>percentage</t>
   </si>
   <si>
-    <t>E-Commerce Sales Analysis Dashboard</t>
-  </si>
-  <si>
     <t>Average Order Value</t>
   </si>
   <si>
@@ -289,10 +187,112 @@
     <t>Total Orders</t>
   </si>
   <si>
-    <t>Tools Used: MySQL, Excel</t>
-  </si>
-  <si>
-    <t>Dataset: Olist Brazilian E-Commerce Dataset (20,000 Orders Sample)</t>
+    <t>Maharashtra</t>
+  </si>
+  <si>
+    <t>Karnataka</t>
+  </si>
+  <si>
+    <t>Tamil Nadu</t>
+  </si>
+  <si>
+    <t>Kerala</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Gujarat</t>
+  </si>
+  <si>
+    <t>Telangana</t>
+  </si>
+  <si>
+    <t>Uttar Pradesh</t>
+  </si>
+  <si>
+    <t>Goa</t>
+  </si>
+  <si>
+    <t>Andhra Pradesh</t>
+  </si>
+  <si>
+    <t>Delhi NCR</t>
+  </si>
+  <si>
+    <t>Punjab</t>
+  </si>
+  <si>
+    <t>Haryana</t>
+  </si>
+  <si>
+    <t>Rajasthan</t>
+  </si>
+  <si>
+    <t>Assam</t>
+  </si>
+  <si>
+    <t>Odisha</t>
+  </si>
+  <si>
+    <t>Bihar</t>
+  </si>
+  <si>
+    <t>Jharkhand</t>
+  </si>
+  <si>
+    <t>Madhya Pradesh</t>
+  </si>
+  <si>
+    <t>Chhattisgarh</t>
+  </si>
+  <si>
+    <t>West Bengal</t>
+  </si>
+  <si>
+    <t>Uttarakhand</t>
+  </si>
+  <si>
+    <t>Himachal Pradesh</t>
+  </si>
+  <si>
+    <t>Health &amp; Beauty</t>
+  </si>
+  <si>
+    <t>Watches &amp; Gifts</t>
+  </si>
+  <si>
+    <t>Sports &amp; Leisure</t>
+  </si>
+  <si>
+    <t>Home &amp; Bedding</t>
+  </si>
+  <si>
+    <t>Electronics &amp; Accessories</t>
+  </si>
+  <si>
+    <t>Furniture &amp; Decor</t>
+  </si>
+  <si>
+    <t>Home Essentials</t>
+  </si>
+  <si>
+    <t>Lifestyle Products</t>
+  </si>
+  <si>
+    <t>Automotive</t>
+  </si>
+  <si>
+    <t>Toys</t>
+  </si>
+  <si>
+    <t>Dataset: Public E-Commerce Dataset adapted for an Indian business scenario</t>
+  </si>
+  <si>
+    <t>Indian E-Commerce Sales Dashboard</t>
+  </si>
+  <si>
+    <t>Tools Used: SQL(MySQL), Excel</t>
   </si>
 </sst>
 </file>
@@ -446,13 +446,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="8" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -467,30 +485,18 @@
     <xf numFmtId="3" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF9BC2E6"/>
+      <color rgb="FF000000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -616,34 +622,34 @@
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>beleza_saude</c:v>
+                  <c:v>Health &amp; Beauty</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>relogios_presentes</c:v>
+                  <c:v>Watches &amp; Gifts</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>esporte_lazer</c:v>
+                  <c:v>Sports &amp; Leisure</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>cama_mesa_banho</c:v>
+                  <c:v>Home &amp; Bedding</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>informatica_acessorios</c:v>
+                  <c:v>Electronics &amp; Accessories</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>moveis_decoracao</c:v>
+                  <c:v>Furniture &amp; Decor</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>utilidades_domesticas</c:v>
+                  <c:v>Home Essentials</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>cool_stuff</c:v>
+                  <c:v>Lifestyle Products</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>automotivo</c:v>
+                  <c:v>Automotive</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>brinquedos</c:v>
+                  <c:v>Toys</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -708,7 +714,7 @@
       <c:catAx>
         <c:axId val="322009711"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -762,7 +768,7 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="t"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -830,10 +836,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="accent1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -1258,10 +1261,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="accent1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -1469,73 +1469,73 @@
               <c:strCache>
                 <c:ptCount val="23"/>
                 <c:pt idx="0">
-                  <c:v>SP</c:v>
+                  <c:v>Maharashtra</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>RJ</c:v>
+                  <c:v>Karnataka</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>MG</c:v>
+                  <c:v>Tamil Nadu</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>SC</c:v>
+                  <c:v>Kerala</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>CE</c:v>
+                  <c:v>Delhi</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>RS</c:v>
+                  <c:v>Gujarat</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>PR</c:v>
+                  <c:v>Telangana</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>BA</c:v>
+                  <c:v>Uttar Pradesh</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>TO</c:v>
+                  <c:v>Goa</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>MA</c:v>
+                  <c:v>Andhra Pradesh</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>SE</c:v>
+                  <c:v>Delhi NCR</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>GO</c:v>
+                  <c:v>Punjab</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>MT</c:v>
+                  <c:v>Haryana</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>MS</c:v>
+                  <c:v>Rajasthan</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>DF</c:v>
+                  <c:v>Assam</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>PE</c:v>
+                  <c:v>Odisha</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>PA</c:v>
+                  <c:v>Bihar</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>PB</c:v>
+                  <c:v>Jharkhand</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>ES</c:v>
+                  <c:v>Madhya Pradesh</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>AL</c:v>
+                  <c:v>Chhattisgarh</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>AM</c:v>
+                  <c:v>West Bengal</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>RN</c:v>
+                  <c:v>Uttarakhand</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>RO</c:v>
+                  <c:v>Himachal Pradesh</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1639,7 +1639,7 @@
       <c:catAx>
         <c:axId val="387147935"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1693,7 +1693,7 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="t"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -2295,7 +2295,7 @@
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="0"/>
+          <c:showLeaderLines val="1"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
         <c:holeSize val="75"/>
@@ -2356,10 +2356,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="accent1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -4048,13 +4045,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>218209</xdr:colOff>
+      <xdr:colOff>218208</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>119842</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>540327</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>361949</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>138545</xdr:rowOff>
     </xdr:to>
@@ -4086,15 +4083,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>221673</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>69273</xdr:rowOff>
+      <xdr:colOff>545522</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>435033</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>153093</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190499</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4124,13 +4121,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>201583</xdr:colOff>
+      <xdr:colOff>201582</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>128154</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>540327</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>400049</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>166254</xdr:rowOff>
     </xdr:to>
@@ -4162,15 +4159,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>261158</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>35329</xdr:rowOff>
+      <xdr:colOff>565959</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>130578</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>498763</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>124691</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190501</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4503,33 +4500,33 @@
     <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1">
         <v>137822.28</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F2" s="1">
         <v>13440</v>
@@ -4537,125 +4534,125 @@
     </row>
     <row r="3" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>74</v>
       </c>
       <c r="B3" s="1">
         <v>113703.37</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="F3" s="1">
         <v>11805</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
+      <c r="A4" t="s">
+        <v>75</v>
       </c>
       <c r="B4" s="1">
         <v>101166.46</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F4" s="1">
         <v>11631.3</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
+      <c r="A5" t="s">
+        <v>76</v>
       </c>
       <c r="B5" s="1">
         <v>97031.07</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="F5" s="1">
         <v>8399.9699999999993</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
+      <c r="A6" t="s">
+        <v>77</v>
       </c>
       <c r="B6" s="1">
         <v>94385.16</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F6" s="1">
         <v>8148</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>5</v>
+      <c r="A7" t="s">
+        <v>78</v>
       </c>
       <c r="B7" s="1">
         <v>88016.45</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F7" s="1">
         <v>8009.73</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>6</v>
+      <c r="A8" t="s">
+        <v>79</v>
       </c>
       <c r="B8" s="1">
         <v>80542.570000000007</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F8" s="1">
         <v>7287.2</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>7</v>
+      <c r="A9" t="s">
+        <v>80</v>
       </c>
       <c r="B9" s="1">
         <v>62545.77</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F9" s="1">
         <v>6735</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
+      <c r="A10" t="s">
+        <v>81</v>
       </c>
       <c r="B10" s="1">
         <v>56175.55</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F10" s="1">
         <v>6428.7</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>9</v>
+      <c r="A11" t="s">
+        <v>82</v>
       </c>
       <c r="B11" s="1">
         <v>53129.09</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F11" s="1">
         <v>6295.8</v>
@@ -4663,27 +4660,27 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E20" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B21" s="1">
         <v>3</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F21" s="1">
         <v>39453.58</v>
@@ -4691,13 +4688,13 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B22" s="1">
         <v>61</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>48</v>
+      <c r="E22" t="s">
+        <v>51</v>
       </c>
       <c r="F22" s="1">
         <v>28645.03</v>
@@ -4705,13 +4702,13 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B23" s="1">
         <v>175</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>49</v>
+      <c r="E23" t="s">
+        <v>52</v>
       </c>
       <c r="F23" s="1">
         <v>11754.82</v>
@@ -4719,13 +4716,13 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B24" s="1">
         <v>350</v>
       </c>
-      <c r="E24" s="1" t="s">
-        <v>50</v>
+      <c r="E24" t="s">
+        <v>53</v>
       </c>
       <c r="F24" s="1">
         <v>8786.35</v>
@@ -4733,13 +4730,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B25" s="1">
         <v>559</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>51</v>
+      <c r="E25" t="s">
+        <v>54</v>
       </c>
       <c r="F25" s="1">
         <v>4233.83</v>
@@ -4747,13 +4744,13 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B26" s="1">
         <v>469</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>52</v>
+      <c r="E26" t="s">
+        <v>55</v>
       </c>
       <c r="F26" s="1">
         <v>3633.82</v>
@@ -4761,13 +4758,13 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B27" s="1">
         <v>752</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>53</v>
+      <c r="E27" t="s">
+        <v>56</v>
       </c>
       <c r="F27" s="1">
         <v>3423.25</v>
@@ -4775,13 +4772,13 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B28" s="1">
         <v>642</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>54</v>
+      <c r="E28" t="s">
+        <v>57</v>
       </c>
       <c r="F28" s="1">
         <v>2859.1</v>
@@ -4789,13 +4786,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B29" s="1">
         <v>797</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>55</v>
+      <c r="E29" t="s">
+        <v>58</v>
       </c>
       <c r="F29" s="1">
         <v>2779.93</v>
@@ -4803,13 +4800,13 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B30" s="1">
         <v>904</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>56</v>
+      <c r="E30" t="s">
+        <v>59</v>
       </c>
       <c r="F30" s="1">
         <v>1631.16</v>
@@ -4817,13 +4814,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B31" s="1">
         <v>843</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>57</v>
+      <c r="E31" t="s">
+        <v>60</v>
       </c>
       <c r="F31" s="1">
         <v>1543.9</v>
@@ -4831,13 +4828,13 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B32" s="1">
         <v>889</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F32" s="1">
         <v>1390.36</v>
@@ -4845,13 +4842,13 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B33" s="1">
         <v>1569</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>59</v>
+      <c r="E33" t="s">
+        <v>62</v>
       </c>
       <c r="F33" s="1">
         <v>1301.57</v>
@@ -4859,13 +4856,13 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B34" s="1">
         <v>1136</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>60</v>
+      <c r="E34" t="s">
+        <v>63</v>
       </c>
       <c r="F34" s="1">
         <v>1027.99</v>
@@ -4873,13 +4870,13 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B35" s="1">
         <v>1451</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F35" s="1">
         <v>936.6</v>
@@ -4887,13 +4884,13 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B36" s="1">
         <v>1385</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F36" s="1">
         <v>876.77</v>
@@ -4901,13 +4898,13 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B37" s="1">
         <v>1443</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>63</v>
+      <c r="E37" t="s">
+        <v>66</v>
       </c>
       <c r="F37" s="1">
         <v>710.69</v>
@@ -4915,13 +4912,13 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B38" s="1">
         <v>1360</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F38" s="1">
         <v>648.9</v>
@@ -4929,13 +4926,13 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B39" s="1">
         <v>1391</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F39" s="1">
         <v>377.8</v>
@@ -4943,13 +4940,13 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B40" s="1">
         <v>1215</v>
       </c>
-      <c r="E40" s="1" t="s">
-        <v>66</v>
+      <c r="E40" t="s">
+        <v>69</v>
       </c>
       <c r="F40" s="1">
         <v>285.29000000000002</v>
@@ -4957,13 +4954,13 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B41" s="1">
         <v>1266</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>67</v>
+      <c r="E41" t="s">
+        <v>70</v>
       </c>
       <c r="F41" s="1">
         <v>214.9</v>
@@ -4971,13 +4968,13 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B42" s="1">
         <v>1336</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>68</v>
+      <c r="E42" t="s">
+        <v>71</v>
       </c>
       <c r="F42" s="1">
         <v>159.97999999999999</v>
@@ -4986,8 +4983,8 @@
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
-      <c r="E43" s="1" t="s">
-        <v>69</v>
+      <c r="E43" t="s">
+        <v>72</v>
       </c>
       <c r="F43" s="1">
         <v>49.9</v>
@@ -4995,18 +4992,18 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="B50" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50" t="s">
         <v>46</v>
-      </c>
-      <c r="C50" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B51" s="1">
         <v>19430</v>
@@ -5017,7 +5014,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="B52" s="1">
         <v>215</v>
@@ -5028,7 +5025,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="B53" s="1">
         <v>124</v>
@@ -5039,7 +5036,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="B54" s="1">
         <v>117</v>
@@ -5050,7 +5047,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="B55" s="1">
         <v>57</v>
@@ -5061,7 +5058,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="B56" s="1">
         <v>55</v>
@@ -5072,7 +5069,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="B57" s="1">
         <v>2</v>
@@ -5082,6 +5079,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B11">
+    <sortCondition descending="1" ref="B2:B11"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5098,36 +5098,36 @@
     <col min="11" max="11" width="19.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+    <row r="1" spans="1:27" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -5149,77 +5149,77 @@
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:27" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A4" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="15"/>
+      <c r="A4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
       <c r="D4" s="4"/>
-      <c r="E4" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="15"/>
+      <c r="E4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="9"/>
+      <c r="G4" s="10"/>
       <c r="H4" s="4"/>
-      <c r="I4" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="J4" s="14"/>
-      <c r="K4" s="15"/>
+      <c r="I4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" s="9"/>
+      <c r="K4" s="10"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
     </row>
     <row r="5" spans="1:27" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A5" s="16"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="8"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="13"/>
       <c r="D5" s="4"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="13"/>
       <c r="H5" s="4"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="8"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="13"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
     <row r="6" spans="1:27" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A6" s="6">
+      <c r="A6" s="14">
         <v>241356.29</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="13"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="12">
+      <c r="E6" s="18">
         <v>20000</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="13"/>
       <c r="H6" s="4"/>
-      <c r="I6" s="6">
+      <c r="I6" s="14">
         <v>137.55000000000001</v>
       </c>
-      <c r="J6" s="7"/>
-      <c r="K6" s="8"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="13"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
     <row r="7" spans="1:27" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="11"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
       <c r="D7" s="4"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="11"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="17"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="11"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="17"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -5853,7 +5853,7 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -5871,7 +5871,7 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>

</xml_diff>